<commit_message>
refactor script: TC-01 - Login
</commit_message>
<xml_diff>
--- a/Data/OpenHRM_Test Data.xlsx
+++ b/Data/OpenHRM_Test Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Katalon Studio\OrangeHRM_TechnicalTest_Azwina_MUF\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25A4D5A9-FB02-42CD-9A1F-964689CF65CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC26AA6-FC48-4ECA-8353-5D0FD32E8CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TC-01_login_page" sheetId="1" r:id="rId1"/>
@@ -710,7 +710,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="13.6640625" customWidth="1"/>
     <col min="4" max="4" width="25.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>